<commit_message>
Earthen Phoenix: note animated services section in links file
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Client-Website-Tracker.xlsx
+++ b/Client-Website-Tracker.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Redesigns" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reports only" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Older previews" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Redesigns" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Reports only" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Older previews" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Redesigns'!$A$1:$O$79</definedName>

</xml_diff>

<commit_message>
Earthen Phoenix: animation layer rebuilt from her practice (Release hero, per-service motions, bowl-ring breath)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Client-Website-Tracker.xlsx
+++ b/Client-Website-Tracker.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Redesigns" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Reports only" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Older previews" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Redesigns" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reports only" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Older previews" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Redesigns'!$A$1:$O$79</definedName>
@@ -6814,7 +6814,7 @@
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>15 Oct 2026</t>
+          <t>15 Oct 2026; 30 Oct 2026 home redesigned; later on 30 Oct 2026 animation layer rebuilt from her practice: full-width photo banner with "Release" (knotted lines loosen under cursor/finger, then breathe), massage pressure ripple on linen + drifting modality tags, yoga line flowing Vinyasa then holding Yin, tappable singing bowl with Reiki light (optional chime, off by default), sprig/constellation/tarot card, bowl-ring breathing circle, root timeline, breath-paced reviews, oil shimmer on products; earth/sand/clay/sage palette, one ember accent; sand garden removed</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Earthen Phoenix: original Ember design preview
New design from scratch (content and photos only carried over); preview copy
in OUTBOX/New/earthenphoenix.com, link in ARTIFACT-LINKS.md, tracker updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Client-Website-Tracker.xlsx
+++ b/Client-Website-Tracker.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Redesigns'!$A$1:$O$80</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Reports only'!$A$1:$D$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Older previews'!$A$1:$D$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Older previews'!$A$1:$D$23</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -561,7 +561,7 @@
         </is>
       </c>
       <c r="B9" s="4" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="11">
@@ -721,12 +721,12 @@
       </c>
       <c r="E2" s="8" t="inlineStr">
         <is>
-          <t>https://claude.ai/artifact/QEntpxndXnFWCdw8vEkJ8o</t>
+          <t>https://claude.ai/artifact/AMnmJyUqsrVg2kgWi25H3x (NEWEST: "Ember", original design)</t>
         </is>
       </c>
       <c r="F2" s="7" t="inlineStr">
         <is>
-          <t>Private until shared (open the link, Share, Anyone with the link). The older home-page link (Jsn9NFxJmciVtundmDbW7H) is public and was not changed.</t>
+          <t>Private until shared (open the link, Share, Anyone with the link)</t>
         </is>
       </c>
       <c r="G2" s="7" t="inlineStr">
@@ -741,19 +741,19 @@
       </c>
       <c r="I2" s="7" t="inlineStr">
         <is>
-          <t>Full 17-page site with per-service animations (30 Oct)</t>
+          <t>Original Ember design, 17 pages, ember service animations (30 Oct)</t>
         </is>
       </c>
       <c r="J2" s="7" t="inlineStr"/>
       <c r="K2" s="7" t="inlineStr"/>
       <c r="L2" s="8" t="inlineStr">
         <is>
-          <t>C:\Users\DaveDeibu\Desktop\VA-KIT\VA-KIT\OUTBOX\New\earthenphoenix.com\2026-10-30_earthenphoenix.com_full-site-preview</t>
+          <t>C:\Users\DaveDeibu\Desktop\VA-KIT\VA-KIT\OUTBOX\New\earthenphoenix.com\2026-10-30_earthenphoenix.com_ember-site-preview</t>
         </is>
       </c>
       <c r="M2" s="7" t="inlineStr">
         <is>
-          <t>Checked 30 Oct (menu panel under header, header pinned after scroll, scrolled header colours)</t>
+          <t>Checked 30 Oct (capsule header stays at top, full-screen menu below it, page locks, links work)</t>
         </is>
       </c>
       <c r="N2" s="7" t="inlineStr">
@@ -6592,7 +6592,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D22"/>
+  <dimension ref="A1:D23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -6869,12 +6869,12 @@
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>Earthen Phoenix full 17-page site (newest; see Website redesigns above)</t>
+          <t>Earthen Phoenix "Ember" original design (newest; see Website redesigns above)</t>
         </is>
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
-          <t>https://claude.ai/artifact/QEntpxndXnFWCdw8vEkJ8o</t>
+          <t>https://claude.ai/artifact/AMnmJyUqsrVg2kgWi25H3x</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
@@ -6889,17 +6889,17 @@
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>Earthen Phoenix (Massage, Yoga &amp; Reiki)</t>
+          <t>Earthen Phoenix full site extending the earlier home design (superseded)</t>
         </is>
       </c>
       <c r="C15" s="8" t="inlineStr">
         <is>
-          <t>https://claude.ai/artifact/Jsn9NFxJmciVtundmDbW7H</t>
+          <t>https://claude.ai/artifact/QEntpxndXnFWCdw8vEkJ8o</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>15 Oct 2026; 30 Oct 2026 home redesigned; later on 30 Oct 2026 animation layer rebuilt from her practice: full-width photo banner with "Release" (knotted lines loosen under cursor/finger, then breathe), massage pressure ripple on linen + drifting modality tags, yoga line flowing Vinyasa then holding Yin, tappable singing bowl with Reiki light (optional chime, off by default), sprig/constellation/tarot card, bowl-ring breathing circle, root timeline, breath-paced reviews, oil shimmer on products; earth/sand/clay/sage palette, one ember accent; sand garden removed; 30 Oct 2026 new page astrology-tarot.html (original design, client example used only as a prompt): star-trail hero over her candle photo, birth-chart wheel that turns to your sun sign, tarot cards with her four steps around a candle that reacts to air, oracle card, teas/rollies/tinctures animations, Oregon to SLC herb journey, $2/min cost meter; facts from her booking page. FLAG: booking page says yoga $140/60 min, home page says $120</t>
+          <t>30 Oct 2026</t>
         </is>
       </c>
     </row>
@@ -6909,17 +6909,17 @@
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>Earthen Phoenix (older)</t>
+          <t>Earthen Phoenix (Massage, Yoga &amp; Reiki)</t>
         </is>
       </c>
       <c r="C16" s="8" t="inlineStr">
         <is>
-          <t>https://claude.ai/artifact/M8XVeqahZEGWSeeqTRxui1</t>
+          <t>https://claude.ai/artifact/Jsn9NFxJmciVtundmDbW7H</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>15 Oct 2026</t>
+          <t>15 Oct 2026; 30 Oct 2026 home redesigned; later on 30 Oct 2026 animation layer rebuilt from her practice: full-width photo banner with "Release" (knotted lines loosen under cursor/finger, then breathe), massage pressure ripple on linen + drifting modality tags, yoga line flowing Vinyasa then holding Yin, tappable singing bowl with Reiki light (optional chime, off by default), sprig/constellation/tarot card, bowl-ring breathing circle, root timeline, breath-paced reviews, oil shimmer on products; earth/sand/clay/sage palette, one ember accent; sand garden removed; 30 Oct 2026 new page astrology-tarot.html (original design, client example used only as a prompt): star-trail hero over her candle photo, birth-chart wheel that turns to your sun sign, tarot cards with her four steps around a candle that reacts to air, oracle card, teas/rollies/tinctures animations, Oregon to SLC herb journey, $2/min cost meter; facts from her booking page. FLAG: booking page says yoga $140/60 min, home page says $120</t>
         </is>
       </c>
     </row>
@@ -6929,17 +6929,17 @@
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>Earthen Phoenix redesign (older)</t>
+          <t>Earthen Phoenix (older)</t>
         </is>
       </c>
       <c r="C17" s="8" t="inlineStr">
         <is>
-          <t>https://claude.ai/artifact/NA6jMpgeLEAc6mMBPQgKpc</t>
+          <t>https://claude.ai/artifact/M8XVeqahZEGWSeeqTRxui1</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>14 Oct 2026</t>
+          <t>15 Oct 2026</t>
         </is>
       </c>
     </row>
@@ -6949,12 +6949,12 @@
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>Alpine Cleaning redesign preview</t>
+          <t>Earthen Phoenix redesign (older)</t>
         </is>
       </c>
       <c r="C18" s="8" t="inlineStr">
         <is>
-          <t>https://claude.ai/artifact/TwW8FzDFCAz6kAQHYPbBLV</t>
+          <t>https://claude.ai/artifact/NA6jMpgeLEAc6mMBPQgKpc</t>
         </is>
       </c>
       <c r="D18" s="7" t="inlineStr">
@@ -6969,12 +6969,12 @@
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>Alpine Cleaning site preview (older)</t>
+          <t>Alpine Cleaning redesign preview</t>
         </is>
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
-          <t>https://claude.ai/artifact/RDm9uD6K7cwSuanyfzVqnT</t>
+          <t>https://claude.ai/artifact/TwW8FzDFCAz6kAQHYPbBLV</t>
         </is>
       </c>
       <c r="D19" s="7" t="inlineStr">
@@ -6989,12 +6989,12 @@
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>Alpine Cleaning preview (older)</t>
+          <t>Alpine Cleaning site preview (older)</t>
         </is>
       </c>
       <c r="C20" s="8" t="inlineStr">
         <is>
-          <t>https://claude.ai/artifact/U6hwEex7gLgva8FFJCJiw6</t>
+          <t>https://claude.ai/artifact/RDm9uD6K7cwSuanyfzVqnT</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
@@ -7009,12 +7009,12 @@
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>Utah Restoration Companies (Water, Fire &amp; Mold)</t>
+          <t>Alpine Cleaning preview (older)</t>
         </is>
       </c>
       <c r="C21" s="8" t="inlineStr">
         <is>
-          <t>https://claude.ai/artifact/ET4zFRQiGsMaT6RPg1bHwd</t>
+          <t>https://claude.ai/artifact/U6hwEex7gLgva8FFJCJiw6</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
@@ -7029,22 +7029,42 @@
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
+          <t>Utah Restoration Companies (Water, Fire &amp; Mold)</t>
+        </is>
+      </c>
+      <c r="C22" s="8" t="inlineStr">
+        <is>
+          <t>https://claude.ai/artifact/ET4zFRQiGsMaT6RPg1bHwd</t>
+        </is>
+      </c>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t>14 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
           <t>The 5-Layer Page Infographic</t>
         </is>
       </c>
-      <c r="C22" s="8" t="inlineStr">
+      <c r="C23" s="8" t="inlineStr">
         <is>
           <t>https://claude.ai/artifact/JfTPtc3pR4ATt1989Qziph</t>
         </is>
       </c>
-      <c r="D22" s="7" t="inlineStr">
+      <c r="D23" s="7" t="inlineStr">
         <is>
           <t>1 Oct 2026</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D22"/>
+  <autoFilter ref="A1:D23"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId2"/>
@@ -7067,6 +7087,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId19"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId20"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId22"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Earthen Phoenix: new original site "The Earthen Atlas" (tension-as-terrain service animations, 17 pages)
Built with the service-animation-website skill. Only words, prices and photos
carried over from earlier drafts. Updates ARTIFACT-LINKS and the tracker.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Client-Website-Tracker.xlsx
+++ b/Client-Website-Tracker.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Redesigns'!$A$1:$O$80</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Reports only'!$A$1:$D$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Older previews'!$A$1:$D$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Older previews'!$A$1:$D$24</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -561,7 +561,7 @@
         </is>
       </c>
       <c r="B9" s="4" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="11">
@@ -711,7 +711,7 @@
       </c>
       <c r="C2" s="7" t="inlineStr">
         <is>
-          <t>Earthen Phoenix</t>
+          <t>Earthen Phoenix, "The Earthen Atlas", newest</t>
         </is>
       </c>
       <c r="D2" s="7" t="inlineStr">
@@ -721,7 +721,7 @@
       </c>
       <c r="E2" s="8" t="inlineStr">
         <is>
-          <t>https://claude.ai/artifact/AMnmJyUqsrVg2kgWi25H3x</t>
+          <t>https://claude.ai/artifact/9Wp2ERpwNbSbJ5LZ7hxGiP</t>
         </is>
       </c>
       <c r="F2" s="7" t="inlineStr">
@@ -731,7 +731,7 @@
       </c>
       <c r="G2" s="7" t="inlineStr">
         <is>
-          <t>30 Oct 2026</t>
+          <t>31 Oct 2026</t>
         </is>
       </c>
       <c r="H2" s="9" t="inlineStr">
@@ -741,24 +741,28 @@
       </c>
       <c r="I2" s="7" t="inlineStr">
         <is>
-          <t>Original Ember design, 17 pages, ember service animations + extra motion layer (30 Oct)</t>
-        </is>
-      </c>
-      <c r="J2" s="7" t="inlineStr"/>
+          <t>New original design "The Earthen Atlas" (31 Oct): tension-as-terrain service animations, 17 pages; replaces Ember (30 Oct)</t>
+        </is>
+      </c>
+      <c r="J2" s="7" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
       <c r="K2" s="7" t="inlineStr"/>
       <c r="L2" s="8" t="inlineStr">
         <is>
-          <t>C:\Users\DaveDeibu\Desktop\VA-KIT\VA-KIT\OUTBOX\New\earthenphoenix.com\2026-10-30_earthenphoenix.com_ember-site-preview</t>
+          <t>C:\Users\DaveDeibu\Desktop\VA-KIT\VA-KIT\OUTBOX\New\earthenphoenix.com\2026-10-31_earthen-phoenix-atlas-website</t>
         </is>
       </c>
       <c r="M2" s="7" t="inlineStr">
         <is>
-          <t>Checked 30 Oct (capsule header stays at top, full-screen menu below it, page locks, links work)</t>
+          <t>Checked 31 Oct (header stays at top 0–64px while scrolling, menu panel starts exactly at the header bottom, page locks, Esc closes; checked at top and after scrolling, home + a session page)</t>
         </is>
       </c>
       <c r="N2" s="7" t="inlineStr">
         <is>
-          <t>client: yoga price ($140 or $120), whether to show the street address and hours, more session photos, OK to reuse the 3 testimonials; developer: move the GHL booking calendar before launch</t>
+          <t>client: yoga price ($140 or $120), whether to show the street address and hours, OK to reuse the 3 testimonials; developer: move the GHL booking calendar before launch, optional real form inbox</t>
         </is>
       </c>
       <c r="O2" s="7" t="inlineStr"/>
@@ -6592,7 +6596,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D23"/>
+  <dimension ref="A1:D24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -6869,17 +6873,17 @@
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>Earthen Phoenix "Ember" original design (newest; see Website redesigns above)</t>
+          <t>Earthen Phoenix "The Earthen Atlas" (newest; see Website redesigns above)</t>
         </is>
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
-          <t>https://claude.ai/artifact/AMnmJyUqsrVg2kgWi25H3x</t>
+          <t>https://claude.ai/artifact/9Wp2ERpwNbSbJ5LZ7hxGiP</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>30 Oct 2026</t>
+          <t>31 Oct 2026</t>
         </is>
       </c>
     </row>
@@ -6889,12 +6893,12 @@
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>Earthen Phoenix full site extending the earlier home design (superseded)</t>
+          <t>Earthen Phoenix "Ember" original design (previous)</t>
         </is>
       </c>
       <c r="C15" s="8" t="inlineStr">
         <is>
-          <t>https://claude.ai/artifact/QEntpxndXnFWCdw8vEkJ8o</t>
+          <t>https://claude.ai/artifact/AMnmJyUqsrVg2kgWi25H3x</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
@@ -6909,17 +6913,17 @@
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>Earthen Phoenix (Massage, Yoga &amp; Reiki)</t>
+          <t>Earthen Phoenix full site extending the earlier home design (superseded)</t>
         </is>
       </c>
       <c r="C16" s="8" t="inlineStr">
         <is>
-          <t>https://claude.ai/artifact/Jsn9NFxJmciVtundmDbW7H</t>
+          <t>https://claude.ai/artifact/QEntpxndXnFWCdw8vEkJ8o</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>15 Oct 2026; 30 Oct 2026 home redesigned; later on 30 Oct 2026 animation layer rebuilt from her practice: full-width photo banner with "Release" (knotted lines loosen under cursor/finger, then breathe), massage pressure ripple on linen + drifting modality tags, yoga line flowing Vinyasa then holding Yin, tappable singing bowl with Reiki light (optional chime, off by default), sprig/constellation/tarot card, bowl-ring breathing circle, root timeline, breath-paced reviews, oil shimmer on products; earth/sand/clay/sage palette, one ember accent; sand garden removed; 30 Oct 2026 new page astrology-tarot.html (original design, client example used only as a prompt): star-trail hero over her candle photo, birth-chart wheel that turns to your sun sign, tarot cards with her four steps around a candle that reacts to air, oracle card, teas/rollies/tinctures animations, Oregon to SLC herb journey, $2/min cost meter; facts from her booking page. FLAG: booking page says yoga $140/60 min, home page says $120</t>
+          <t>30 Oct 2026</t>
         </is>
       </c>
     </row>
@@ -6929,17 +6933,17 @@
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>Earthen Phoenix (older)</t>
+          <t>Earthen Phoenix (Massage, Yoga &amp; Reiki)</t>
         </is>
       </c>
       <c r="C17" s="8" t="inlineStr">
         <is>
-          <t>https://claude.ai/artifact/M8XVeqahZEGWSeeqTRxui1</t>
+          <t>https://claude.ai/artifact/Jsn9NFxJmciVtundmDbW7H</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>15 Oct 2026</t>
+          <t>15 Oct 2026; 30 Oct 2026 home redesigned; later on 30 Oct 2026 animation layer rebuilt from her practice: full-width photo banner with "Release" (knotted lines loosen under cursor/finger, then breathe), massage pressure ripple on linen + drifting modality tags, yoga line flowing Vinyasa then holding Yin, tappable singing bowl with Reiki light (optional chime, off by default), sprig/constellation/tarot card, bowl-ring breathing circle, root timeline, breath-paced reviews, oil shimmer on products; earth/sand/clay/sage palette, one ember accent; sand garden removed; 30 Oct 2026 new page astrology-tarot.html (original design, client example used only as a prompt): star-trail hero over her candle photo, birth-chart wheel that turns to your sun sign, tarot cards with her four steps around a candle that reacts to air, oracle card, teas/rollies/tinctures animations, Oregon to SLC herb journey, $2/min cost meter; facts from her booking page. FLAG: booking page says yoga $140/60 min, home page says $120</t>
         </is>
       </c>
     </row>
@@ -6949,17 +6953,17 @@
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>Earthen Phoenix redesign (older)</t>
+          <t>Earthen Phoenix (older)</t>
         </is>
       </c>
       <c r="C18" s="8" t="inlineStr">
         <is>
-          <t>https://claude.ai/artifact/NA6jMpgeLEAc6mMBPQgKpc</t>
+          <t>https://claude.ai/artifact/M8XVeqahZEGWSeeqTRxui1</t>
         </is>
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>14 Oct 2026</t>
+          <t>15 Oct 2026</t>
         </is>
       </c>
     </row>
@@ -6969,12 +6973,12 @@
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>Alpine Cleaning redesign preview</t>
+          <t>Earthen Phoenix redesign (older)</t>
         </is>
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
-          <t>https://claude.ai/artifact/TwW8FzDFCAz6kAQHYPbBLV</t>
+          <t>https://claude.ai/artifact/NA6jMpgeLEAc6mMBPQgKpc</t>
         </is>
       </c>
       <c r="D19" s="7" t="inlineStr">
@@ -6989,12 +6993,12 @@
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>Alpine Cleaning site preview (older)</t>
+          <t>Alpine Cleaning redesign preview</t>
         </is>
       </c>
       <c r="C20" s="8" t="inlineStr">
         <is>
-          <t>https://claude.ai/artifact/RDm9uD6K7cwSuanyfzVqnT</t>
+          <t>https://claude.ai/artifact/TwW8FzDFCAz6kAQHYPbBLV</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
@@ -7009,12 +7013,12 @@
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>Alpine Cleaning preview (older)</t>
+          <t>Alpine Cleaning site preview (older)</t>
         </is>
       </c>
       <c r="C21" s="8" t="inlineStr">
         <is>
-          <t>https://claude.ai/artifact/U6hwEex7gLgva8FFJCJiw6</t>
+          <t>https://claude.ai/artifact/RDm9uD6K7cwSuanyfzVqnT</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
@@ -7029,12 +7033,12 @@
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>Utah Restoration Companies (Water, Fire &amp; Mold)</t>
+          <t>Alpine Cleaning preview (older)</t>
         </is>
       </c>
       <c r="C22" s="8" t="inlineStr">
         <is>
-          <t>https://claude.ai/artifact/ET4zFRQiGsMaT6RPg1bHwd</t>
+          <t>https://claude.ai/artifact/U6hwEex7gLgva8FFJCJiw6</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
@@ -7049,22 +7053,42 @@
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
+          <t>Utah Restoration Companies (Water, Fire &amp; Mold)</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>https://claude.ai/artifact/ET4zFRQiGsMaT6RPg1bHwd</t>
+        </is>
+      </c>
+      <c r="D23" s="7" t="inlineStr">
+        <is>
+          <t>14 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="7" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
           <t>The 5-Layer Page Infographic</t>
         </is>
       </c>
-      <c r="C23" s="8" t="inlineStr">
+      <c r="C24" s="8" t="inlineStr">
         <is>
           <t>https://claude.ai/artifact/JfTPtc3pR4ATt1989Qziph</t>
         </is>
       </c>
-      <c r="D23" s="7" t="inlineStr">
+      <c r="D24" s="7" t="inlineStr">
         <is>
           <t>1 Oct 2026</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D23"/>
+  <autoFilter ref="A1:D24"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId2"/>
@@ -7088,6 +7112,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId20"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId21"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId23"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>